<commit_message>
Registrar faltantes Req_003_ULOP · A-2510-K100188-61401-D/0528/2021
</commit_message>
<xml_diff>
--- a/data/Documentacion_faltante.xlsx
+++ b/data/Documentacion_faltante.xlsx
@@ -919,7 +919,12 @@
           <t>URBANIZADORA Y CONSTRUCTORA CURG SA DE CV</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n"/>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Bitácora de obra
+Finiquito (excel)</t>
+        </is>
+      </c>
       <c r="F8" s="11" t="n"/>
     </row>
     <row r="9" ht="60" customHeight="1">
@@ -3541,7 +3546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3676,6 +3681,96 @@
         </is>
       </c>
       <c r="I3" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>48ae1d348d0d4e2bacf20a1150ca358e</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Req_003_ULOP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A-2510-K100188-61401-D/0528/2021</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>DIR</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>EJE_DIR_BIT.pdf</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Bitácora de obra</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="n">
+        <v>46255.63350694445</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>LFAM</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>03e897659f094577882a0c7fb88e54f6</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Req_003_ULOP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A-2510-K100188-61401-D/0528/2021</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DIR</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ETR_DIR_FIN.xls</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Finiquito (excel)</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="n">
+        <v>46255.63350694445</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>LFAM</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>

</xml_diff>

<commit_message>
Registrar faltantes Req_003_ULOP · G-5051-K100250-61401-D/0541/2022
</commit_message>
<xml_diff>
--- a/data/Documentacion_faltante.xlsx
+++ b/data/Documentacion_faltante.xlsx
@@ -1051,7 +1051,11 @@
           <t>CONSTRUCCION Y SERVICIOS DEL BAJIO SA DE CV</t>
         </is>
       </c>
-      <c r="E13" s="12" t="n"/>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Normas de calidad</t>
+        </is>
+      </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
           <t>XGOT</t>
@@ -3548,7 +3552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3768,6 +3772,51 @@
       </c>
       <c r="I5" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>c950cb7776c742df8e0c118f12c38e61</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Req_003_ULOP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>G-5051-K100250-61401-D/0541/2022</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DIR</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PPP_DIR_NOC.pdf</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Normas de calidad</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="n">
+        <v>46255.68847222222</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>XGOT</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Registrar faltantes Req_003_ULOP · GD-564023
</commit_message>
<xml_diff>
--- a/data/Documentacion_faltante.xlsx
+++ b/data/Documentacion_faltante.xlsx
@@ -3553,7 +3553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3860,6 +3860,51 @@
         </is>
       </c>
       <c r="I7" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9fced7554a224c71b5e4b959356ad4e2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Req_003_ULOP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GD-564023</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DIR</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PPP_DIR_EIA.pdf</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Estudios de factibilidad y evaluación de impacto ambiental</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="n">
+        <v>46261.12668981482</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>DAPF</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>

</xml_diff>

<commit_message>
Retirar documentos Corte 1 · Req_003_ULOP
</commit_message>
<xml_diff>
--- a/data/Documentacion_faltante.xlsx
+++ b/data/Documentacion_faltante.xlsx
@@ -3553,7 +3553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3602,6 +3602,11 @@
           <t>Corte</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Especificacion</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3771,8 +3776,10 @@
           <t>LFAM</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>1</v>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3979,7 +3986,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Eliminar faltantes pendientes · Req_003_ULOP
</commit_message>
<xml_diff>
--- a/data/Documentacion_faltante.xlsx
+++ b/data/Documentacion_faltante.xlsx
@@ -3553,7 +3553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3867,51 +3867,6 @@
         </is>
       </c>
       <c r="I7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>9fced7554a224c71b5e4b959356ad4e2</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Req_003_ULOP</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>GD-564023</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>DIR</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PPP_DIR_EIA.pdf</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Estudios de factibilidad y evaluación de impacto ambiental</t>
-        </is>
-      </c>
-      <c r="G8" s="28" t="n">
-        <v>46261.12668981482</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>DAPF</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
         </is>

</xml_diff>

<commit_message>
Eliminar Corte 1 · Req_003_ULOP
</commit_message>
<xml_diff>
--- a/data/Documentacion_faltante.xlsx
+++ b/data/Documentacion_faltante.xlsx
@@ -3647,8 +3647,10 @@
           <t>DAPF</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>1</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -3690,8 +3692,10 @@
           <t>DAPF</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>1</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -3733,8 +3737,10 @@
           <t>LFAM</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>1</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -3883,7 +3889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3916,32 +3922,6 @@
         <is>
           <t>Documentos</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>e59b21be404944e7bebd999797e37d83</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Req_003_ULOP</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="29" t="n">
-        <v>46255</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>LFAM</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Eliminar Corte 2 · Req_003_ULOP
</commit_message>
<xml_diff>
--- a/data/Documentacion_faltante.xlsx
+++ b/data/Documentacion_faltante.xlsx
@@ -3691,8 +3691,10 @@
           <t>XGOT</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>2</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -3734,8 +3736,10 @@
           <t>DAPF</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>2</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3749,7 +3753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3782,32 +3786,6 @@
         <is>
           <t>Documentos</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>eab137135eed4496856f73e34e7f4fe9</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Req_003_ULOP</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" s="29" t="n">
-        <v>46261</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>LFAM</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>